<commit_message>
Synchronize final Biology Open submission package
</commit_message>
<xml_diff>
--- a/Table_S12.xlsx
+++ b/Table_S12.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12_seed_variants" sheetId="1" r:id="R688e74111dc84719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12_seed_variants" sheetId="1" r:id="R6471ff1080a445e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -217,9 +217,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -339,15 +339,15 @@
       <x:c r="A1" s="22" t="str">
         <x:v>Table S12. Natural 49-bp ONSEN-like HSE seed-variant accession summary.</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="n"/>
-      <x:c r="C1" s="1" t="n"/>
-      <x:c r="D1" s="1" t="n"/>
-      <x:c r="E1" s="1" t="n"/>
-      <x:c r="F1" s="1" t="n"/>
-      <x:c r="G1" s="1" t="n"/>
-      <x:c r="H1" s="1" t="n"/>
-      <x:c r="I1" s="1" t="n"/>
-      <x:c r="J1" s="1" t="n"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Synchronize final S1-S13 revision package
</commit_message>
<xml_diff>
--- a/Table_S12.xlsx
+++ b/Table_S12.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12_seed_variants" sheetId="1" r:id="R688e74111dc84719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12_seed_variants" sheetId="1" r:id="R6471ff1080a445e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -217,9 +217,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -339,15 +339,15 @@
       <x:c r="A1" s="22" t="str">
         <x:v>Table S12. Natural 49-bp ONSEN-like HSE seed-variant accession summary.</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="n"/>
-      <x:c r="C1" s="1" t="n"/>
-      <x:c r="D1" s="1" t="n"/>
-      <x:c r="E1" s="1" t="n"/>
-      <x:c r="F1" s="1" t="n"/>
-      <x:c r="G1" s="1" t="n"/>
-      <x:c r="H1" s="1" t="n"/>
-      <x:c r="I1" s="1" t="n"/>
-      <x:c r="J1" s="1" t="n"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="inlineStr">

</xml_diff>